<commit_message>
chore: limpieza — borrar archivos duplicados y backups viejos
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bancos_paquetes_tarjetas.xlsx
+++ b/bancos_paquetes_tarjetas.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Proyectos\promoar\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\Proyectos\promoar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90B106A3-52AE-4D90-B108-37E13319CDF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4F673A9-4F61-4E02-BBF4-DDAAD0230C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DFF26E67-F130-4B3A-A60D-D784D61A921C}"/>
+    <workbookView xWindow="-25320" yWindow="1995" windowWidth="25440" windowHeight="15390" xr2:uid="{DFF26E67-F130-4B3A-A60D-D784D61A921C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Hoja2!$A$1:$N$90</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="136">
   <si>
     <t>Visa Debito</t>
   </si>
@@ -434,6 +436,21 @@
   </si>
   <si>
     <t>Plan Ultra</t>
+  </si>
+  <si>
+    <t>Mastercard Credito Black</t>
+  </si>
+  <si>
+    <t>Macro Selecta Signature</t>
+  </si>
+  <si>
+    <t>Macro Selecta Black</t>
+  </si>
+  <si>
+    <t>Macro Selecta Icon</t>
+  </si>
+  <si>
+    <t>Bco Santa Cruz</t>
   </si>
 </sst>
 </file>
@@ -457,12 +474,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -477,10 +500,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -499,7 +523,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -816,21 +840,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3A49304-E782-4629-961F-5A561024EF18}">
   <dimension ref="A1:S113"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.36328125" customWidth="1"/>
+    <col min="3" max="3" width="23.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>119</v>
       </c>
@@ -877,7 +901,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>105</v>
       </c>
@@ -897,23 +921,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="R3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="R4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="R5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B6" t="s">
@@ -922,6 +946,9 @@
       <c r="C6" t="s">
         <v>44</v>
       </c>
+      <c r="D6" t="s">
+        <v>135</v>
+      </c>
       <c r="E6" t="s">
         <v>44</v>
       </c>
@@ -932,7 +959,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A7" s="3"/>
       <c r="B7" t="s">
         <v>5</v>
       </c>
@@ -946,7 +974,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A8" s="3"/>
       <c r="B8" t="s">
         <v>6</v>
       </c>
@@ -957,7 +986,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A9" s="3"/>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A10" s="3"/>
       <c r="R10" t="s">
         <v>15</v>
       </c>
@@ -965,8 +998,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B11" t="s">
@@ -982,7 +1015,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A12" s="3"/>
       <c r="B12" t="s">
         <v>13</v>
       </c>
@@ -996,7 +1030,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A13" s="3"/>
       <c r="B13" t="s">
         <v>14</v>
       </c>
@@ -1010,7 +1045,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A14" s="3"/>
       <c r="B14" t="s">
         <v>15</v>
       </c>
@@ -1021,7 +1057,8 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A15" s="3"/>
       <c r="B15" t="s">
         <v>16</v>
       </c>
@@ -1029,8 +1066,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B16" t="s">
@@ -1049,7 +1086,8 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A17" s="3"/>
       <c r="B17" t="s">
         <v>13</v>
       </c>
@@ -1060,7 +1098,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A18" s="3"/>
       <c r="B18" t="s">
         <v>14</v>
       </c>
@@ -1071,7 +1110,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A19" s="3"/>
       <c r="B19" t="s">
         <v>15</v>
       </c>
@@ -1082,13 +1122,14 @@
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A20" s="3"/>
       <c r="B20" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A21" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B21" t="s">
@@ -1097,27 +1138,33 @@
       <c r="C21" t="s">
         <v>60</v>
       </c>
+      <c r="D21" t="s">
+        <v>0</v>
+      </c>
       <c r="G21" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A22" s="3"/>
       <c r="B22" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A23" s="3"/>
       <c r="B23" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A24" s="3"/>
       <c r="B24" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A25" s="3" t="s">
         <v>106</v>
       </c>
       <c r="B25" t="s">
@@ -1139,7 +1186,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A26" s="3"/>
       <c r="C26" t="s">
         <v>46</v>
       </c>
@@ -1150,7 +1198,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A27" s="3"/>
       <c r="C27" t="s">
         <v>45</v>
       </c>
@@ -1158,7 +1207,8 @@
         <v>120</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A28" s="3"/>
       <c r="C28" t="s">
         <v>44</v>
       </c>
@@ -1166,13 +1216,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A29" s="3"/>
       <c r="C29" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A30" s="3" t="s">
         <v>30</v>
       </c>
       <c r="B30" t="s">
@@ -1188,7 +1239,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A31" s="3"/>
       <c r="B31" t="s">
         <v>33</v>
       </c>
@@ -1199,7 +1251,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A32" s="3"/>
       <c r="B32" t="s">
         <v>34</v>
       </c>
@@ -1210,7 +1263,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A33" s="3"/>
       <c r="B33" t="s">
         <v>35</v>
       </c>
@@ -1221,13 +1275,14 @@
         <v>46</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A34" s="3"/>
       <c r="B34" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A35" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B35" t="s">
@@ -1243,7 +1298,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A36" s="3"/>
       <c r="B36" t="s">
         <v>33</v>
       </c>
@@ -1254,7 +1310,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A37" s="3"/>
       <c r="B37" t="s">
         <v>34</v>
       </c>
@@ -1265,7 +1322,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A38" s="3"/>
       <c r="B38" t="s">
         <v>35</v>
       </c>
@@ -1276,13 +1334,14 @@
         <v>46</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A39" s="3"/>
       <c r="B39" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A40" s="3" t="s">
         <v>38</v>
       </c>
       <c r="B40" t="s">
@@ -1301,7 +1360,8 @@
         <v>43</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A41" s="3"/>
       <c r="B41" t="s">
         <v>34</v>
       </c>
@@ -1315,7 +1375,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A42" s="3"/>
       <c r="B42" t="s">
         <v>40</v>
       </c>
@@ -1329,7 +1390,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A43" s="3"/>
       <c r="C43" t="s">
         <v>46</v>
       </c>
@@ -1340,8 +1402,8 @@
         <v>46</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A44" s="3" t="s">
         <v>107</v>
       </c>
       <c r="B44" t="s">
@@ -1365,7 +1427,8 @@
         <v>121</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A45" s="3"/>
       <c r="B45" t="s">
         <v>51</v>
       </c>
@@ -1385,7 +1448,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A46" s="3"/>
       <c r="B46" t="s">
         <v>49</v>
       </c>
@@ -1405,7 +1469,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A47" s="3"/>
       <c r="B47" t="s">
         <v>50</v>
       </c>
@@ -1425,7 +1490,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A48" s="3"/>
       <c r="B48" t="s">
         <v>44</v>
       </c>
@@ -1439,7 +1505,8 @@
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A49" s="3"/>
       <c r="B49" t="s">
         <v>42</v>
       </c>
@@ -1453,8 +1520,8 @@
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A50" s="3" t="s">
         <v>52</v>
       </c>
       <c r="B50" t="s">
@@ -1476,7 +1543,8 @@
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A51" s="3"/>
       <c r="B51" t="s">
         <v>54</v>
       </c>
@@ -1494,7 +1562,8 @@
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A52" s="3"/>
       <c r="B52" t="s">
         <v>55</v>
       </c>
@@ -1512,7 +1581,8 @@
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A53" s="3"/>
       <c r="B53" t="s">
         <v>56</v>
       </c>
@@ -1530,8 +1600,8 @@
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A54" s="3" t="s">
         <v>108</v>
       </c>
       <c r="B54" t="s">
@@ -1557,7 +1627,8 @@
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A55" s="3"/>
       <c r="B55" t="s">
         <v>58</v>
       </c>
@@ -1575,7 +1646,8 @@
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A56" s="3"/>
       <c r="B56" t="s">
         <v>59</v>
       </c>
@@ -1593,7 +1665,8 @@
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A57" s="3"/>
       <c r="C57" s="2" t="s">
         <v>41</v>
       </c>
@@ -1608,8 +1681,8 @@
       <c r="J57" s="2"/>
       <c r="K57" s="2"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A58" s="3" t="s">
         <v>109</v>
       </c>
       <c r="B58" t="s">
@@ -1633,7 +1706,8 @@
         <v>65</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A59" s="3"/>
       <c r="C59" s="2" t="s">
         <v>45</v>
       </c>
@@ -1650,7 +1724,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A60" s="3"/>
       <c r="C60" s="2" t="s">
         <v>44</v>
       </c>
@@ -1667,7 +1742,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A61" s="3"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
       <c r="E61" s="2"/>
@@ -1678,8 +1754,8 @@
       <c r="J61" s="2"/>
       <c r="K61" s="2"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A62" s="3" t="s">
         <v>110</v>
       </c>
       <c r="B62" t="s">
@@ -1701,7 +1777,8 @@
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A63" s="3"/>
       <c r="B63" t="s">
         <v>123</v>
       </c>
@@ -1719,7 +1796,8 @@
       <c r="J63" s="2"/>
       <c r="K63" s="2"/>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A64" s="3"/>
       <c r="B64" t="s">
         <v>124</v>
       </c>
@@ -1737,7 +1815,8 @@
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A65" s="3"/>
       <c r="B65" t="s">
         <v>125</v>
       </c>
@@ -1748,8 +1827,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A66" s="3" t="s">
         <v>111</v>
       </c>
       <c r="B66" t="s">
@@ -1771,7 +1850,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A67" s="3"/>
       <c r="B67" t="s">
         <v>68</v>
       </c>
@@ -1782,7 +1862,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A68" s="3"/>
       <c r="B68" t="s">
         <v>69</v>
       </c>
@@ -1793,7 +1874,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A69" s="3"/>
       <c r="B69" t="s">
         <v>70</v>
       </c>
@@ -1804,8 +1886,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A70" s="3" t="s">
         <v>112</v>
       </c>
       <c r="B70" t="s">
@@ -1821,7 +1903,8 @@
         <v>46</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A71" s="3"/>
       <c r="B71" t="s">
         <v>44</v>
       </c>
@@ -1832,7 +1915,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A72" s="3"/>
       <c r="B72" t="s">
         <v>72</v>
       </c>
@@ -1843,7 +1927,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A73" s="3"/>
       <c r="C73" t="s">
         <v>41</v>
       </c>
@@ -1851,8 +1936,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A74" s="3" t="s">
         <v>73</v>
       </c>
       <c r="B74" t="s">
@@ -1868,7 +1953,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A75" s="3"/>
       <c r="B75" t="s">
         <v>34</v>
       </c>
@@ -1879,7 +1965,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A76" s="3"/>
       <c r="B76" t="s">
         <v>60</v>
       </c>
@@ -1890,7 +1977,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A77" s="3"/>
       <c r="C77" t="s">
         <v>46</v>
       </c>
@@ -1898,13 +1986,14 @@
         <v>46</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A78" s="3"/>
       <c r="C78" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A79" s="3" t="s">
         <v>113</v>
       </c>
       <c r="B79" t="s">
@@ -1920,7 +2009,8 @@
         <v>46</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A80" s="3"/>
       <c r="B80" t="s">
         <v>77</v>
       </c>
@@ -1934,7 +2024,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A81" s="3"/>
       <c r="B81" t="s">
         <v>78</v>
       </c>
@@ -1945,13 +2036,14 @@
         <v>79</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A82" s="3"/>
       <c r="C82" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A83" s="3" t="s">
         <v>114</v>
       </c>
       <c r="B83" t="s">
@@ -1961,8 +2053,8 @@
         <v>46</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A84" s="3" t="s">
         <v>115</v>
       </c>
       <c r="B84" t="s">
@@ -1978,7 +2070,8 @@
         <v>46</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A85" s="3"/>
       <c r="B85" t="s">
         <v>81</v>
       </c>
@@ -1989,7 +2082,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A86" s="3"/>
       <c r="B86" t="s">
         <v>82</v>
       </c>
@@ -2000,7 +2094,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A87" s="3"/>
       <c r="B87" t="s">
         <v>83</v>
       </c>
@@ -2011,8 +2106,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A88" t="s">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A88" s="3" t="s">
         <v>116</v>
       </c>
       <c r="B88" t="s">
@@ -2025,7 +2120,8 @@
         <v>47</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A89" s="3"/>
       <c r="B89" s="2" t="s">
         <v>85</v>
       </c>
@@ -2033,7 +2129,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A90" s="3"/>
       <c r="B90" s="2" t="s">
         <v>86</v>
       </c>
@@ -2041,7 +2138,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A91" s="3"/>
       <c r="B91" s="2" t="s">
         <v>87</v>
       </c>
@@ -2049,23 +2147,26 @@
         <v>41</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A92" s="3"/>
       <c r="B92" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A93" s="3"/>
       <c r="B93" s="2" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A94" s="3"/>
       <c r="B94" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A96" s="3" t="s">
         <v>117</v>
       </c>
       <c r="B96" t="s">
@@ -2084,7 +2185,8 @@
         <v>46</v>
       </c>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A97" s="3"/>
       <c r="B97" t="s">
         <v>95</v>
       </c>
@@ -2098,7 +2200,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A98" s="3"/>
       <c r="B98" t="s">
         <v>93</v>
       </c>
@@ -2112,23 +2215,26 @@
         <v>42</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A99" s="3"/>
       <c r="B99" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A100" s="3"/>
       <c r="B100" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A101" s="3"/>
       <c r="B101" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A102" t="s">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A102" s="3" t="s">
         <v>118</v>
       </c>
       <c r="B102" t="s">
@@ -2138,18 +2244,23 @@
         <v>60</v>
       </c>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A103" s="3"/>
       <c r="B103" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A104" s="3"/>
       <c r="B104" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A106" t="s">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A105" s="3"/>
+    </row>
+    <row r="106" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A106" s="3" t="s">
         <v>97</v>
       </c>
       <c r="B106" t="s">
@@ -2165,40 +2276,45 @@
         <v>97</v>
       </c>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A107" t="s">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A107" s="3" t="s">
         <v>27</v>
       </c>
       <c r="K107" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A108" s="3"/>
       <c r="K108" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A109" s="3"/>
       <c r="K109" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A110" s="3"/>
       <c r="K110" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A111" s="3"/>
       <c r="K111" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A112" s="3"/>
       <c r="K112" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A113" s="1"/>
     </row>
   </sheetData>
@@ -2209,20 +2325,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{871C37FC-D831-4651-AA0B-2C8C35015B53}">
   <dimension ref="A1:R91"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.81640625" customWidth="1"/>
+    <col min="2" max="2" width="23.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.08984375" customWidth="1"/>
+    <col min="4" max="4" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>119</v>
       </c>
@@ -2266,7 +2382,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>105</v>
       </c>
@@ -2274,24 +2390,24 @@
         <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="Q2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>44</v>
       </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="Q3" t="s">
         <v>3</v>
@@ -2300,32 +2416,41 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>45</v>
       </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="Q4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2</v>
       </c>
       <c r="B5" t="s">
         <v>46</v>
       </c>
+      <c r="C5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" t="s">
+        <v>42</v>
+      </c>
       <c r="Q5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2339,7 +2464,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2353,7 +2478,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2367,7 +2492,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2378,7 +2503,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -2395,7 +2520,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -2406,7 +2531,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -2417,7 +2542,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -2428,7 +2553,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -2439,22 +2564,22 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>106</v>
       </c>
@@ -2474,7 +2599,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>106</v>
       </c>
@@ -2488,7 +2613,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>106</v>
       </c>
@@ -2499,7 +2624,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>106</v>
       </c>
@@ -2510,7 +2635,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>106</v>
       </c>
@@ -2518,7 +2643,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -2532,7 +2657,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -2543,7 +2668,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -2554,7 +2679,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -2565,7 +2690,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -2579,7 +2704,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -2590,7 +2715,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>37</v>
       </c>
@@ -2601,7 +2726,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>37</v>
       </c>
@@ -2612,7 +2737,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>38</v>
       </c>
@@ -2629,7 +2754,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>38</v>
       </c>
@@ -2643,7 +2768,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>38</v>
       </c>
@@ -2657,7 +2782,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -2667,11 +2792,8 @@
       <c r="D34" t="s">
         <v>46</v>
       </c>
-      <c r="J34" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>107</v>
       </c>
@@ -2689,11 +2811,9 @@
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
-      <c r="J35" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J35" s="2"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>107</v>
       </c>
@@ -2713,7 +2833,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>107</v>
       </c>
@@ -2733,7 +2853,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>107</v>
       </c>
@@ -2750,10 +2870,10 @@
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>52</v>
       </c>
@@ -2773,7 +2893,7 @@
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>52</v>
       </c>
@@ -2791,7 +2911,7 @@
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>52</v>
       </c>
@@ -2809,7 +2929,7 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>52</v>
       </c>
@@ -2827,7 +2947,7 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>108</v>
       </c>
@@ -2851,7 +2971,7 @@
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>108</v>
       </c>
@@ -2869,7 +2989,7 @@
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>108</v>
       </c>
@@ -2887,7 +3007,7 @@
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>108</v>
       </c>
@@ -2905,18 +3025,18 @@
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>109</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>65</v>
+        <v>132</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>47</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>65</v>
+        <v>133</v>
       </c>
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
@@ -2924,10 +3044,10 @@
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>109</v>
       </c>
@@ -2947,7 +3067,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>109</v>
       </c>
@@ -2967,7 +3087,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>110</v>
       </c>
@@ -2987,7 +3107,7 @@
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>110</v>
       </c>
@@ -3005,7 +3125,7 @@
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>110</v>
       </c>
@@ -3023,7 +3143,7 @@
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>110</v>
       </c>
@@ -3034,7 +3154,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>111</v>
       </c>
@@ -3054,7 +3174,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>111</v>
       </c>
@@ -3065,7 +3185,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>111</v>
       </c>
@@ -3076,7 +3196,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>111</v>
       </c>
@@ -3087,7 +3207,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>112</v>
       </c>
@@ -3101,7 +3221,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>112</v>
       </c>
@@ -3112,7 +3232,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>112</v>
       </c>
@@ -3123,7 +3243,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>112</v>
       </c>
@@ -3134,7 +3254,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>73</v>
       </c>
@@ -3148,7 +3268,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>73</v>
       </c>
@@ -3159,7 +3279,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>73</v>
       </c>
@@ -3170,7 +3290,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>73</v>
       </c>
@@ -3181,7 +3301,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>73</v>
       </c>
@@ -3189,7 +3309,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>113</v>
       </c>
@@ -3203,7 +3323,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>113</v>
       </c>
@@ -3217,7 +3337,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>113</v>
       </c>
@@ -3228,7 +3348,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>113</v>
       </c>
@@ -3236,7 +3356,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>114</v>
       </c>
@@ -3244,7 +3364,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>115</v>
       </c>
@@ -3258,7 +3378,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>115</v>
       </c>
@@ -3269,7 +3389,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>115</v>
       </c>
@@ -3280,7 +3400,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>115</v>
       </c>
@@ -3291,7 +3411,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>116</v>
       </c>
@@ -3302,7 +3422,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>116</v>
       </c>
@@ -3310,7 +3430,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>116</v>
       </c>
@@ -3318,7 +3438,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>116</v>
       </c>
@@ -3326,7 +3446,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>117</v>
       </c>
@@ -3339,11 +3459,8 @@
       <c r="D80" t="s">
         <v>46</v>
       </c>
-      <c r="J80" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>117</v>
       </c>
@@ -3357,7 +3474,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>117</v>
       </c>
@@ -3368,10 +3485,10 @@
         <v>42</v>
       </c>
       <c r="J82" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>118</v>
       </c>
@@ -3379,7 +3496,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>97</v>
       </c>
@@ -3393,7 +3510,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>27</v>
       </c>
@@ -3401,7 +3518,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>27</v>
       </c>
@@ -3409,7 +3526,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>27</v>
       </c>
@@ -3417,7 +3534,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>27</v>
       </c>
@@ -3425,7 +3542,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>27</v>
       </c>
@@ -3433,7 +3550,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>27</v>
       </c>
@@ -3441,10 +3558,11 @@
         <v>103</v>
       </c>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A91" s="1"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:N90" xr:uid="{871C37FC-D831-4651-AA0B-2C8C35015B53}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>